<commit_message>
Melhoria de README + atualização requirements
</commit_message>
<xml_diff>
--- a/src/Referencia_Variaveis/Importancia_Variaveis_CH.xlsx
+++ b/src/Referencia_Variaveis/Importancia_Variaveis_CH.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Armazenamento\MBA\TCC\TccMbaUspEsalq\src\Referencia_Variaveis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95F3E763-FC33-43AC-9B66-3396DCC18D2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3BED4A8-F46E-47BC-99AA-6E14ACE9F42D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -157,9 +157,6 @@
     <t>Qtde. carros</t>
   </si>
   <si>
-    <t>Dias empregado(a) doméstico(a)</t>
-  </si>
-  <si>
     <t>Educação profissional</t>
   </si>
   <si>
@@ -359,6 +356,9 @@
   </si>
   <si>
     <t>Ocupação galpão</t>
+  </si>
+  <si>
+    <t>Qtde. de Dias empregado(a)</t>
   </si>
 </sst>
 </file>
@@ -1397,7 +1397,7 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>45</v>
+        <v>112</v>
       </c>
       <c r="B40" t="s">
         <v>6</v>
@@ -1414,7 +1414,7 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B41" t="s">
         <v>14</v>
@@ -1431,7 +1431,7 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B42" t="s">
         <v>14</v>
@@ -1448,7 +1448,7 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B43" t="s">
         <v>6</v>
@@ -1465,7 +1465,7 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B44" t="s">
         <v>14</v>
@@ -1482,7 +1482,7 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B45" t="s">
         <v>14</v>
@@ -1499,7 +1499,7 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B46" t="s">
         <v>14</v>
@@ -1516,7 +1516,7 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B47" t="s">
         <v>6</v>
@@ -1533,7 +1533,7 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B48" t="s">
         <v>14</v>
@@ -1550,7 +1550,7 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B49" t="s">
         <v>14</v>
@@ -1567,7 +1567,7 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B50" t="s">
         <v>6</v>
@@ -1584,7 +1584,7 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B51" t="s">
         <v>6</v>
@@ -1601,7 +1601,7 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B52" t="s">
         <v>14</v>
@@ -1618,7 +1618,7 @@
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B53" t="s">
         <v>14</v>
@@ -1635,7 +1635,7 @@
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B54" t="s">
         <v>14</v>
@@ -1652,7 +1652,7 @@
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B55" t="s">
         <v>6</v>
@@ -1669,7 +1669,7 @@
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B56" t="s">
         <v>14</v>
@@ -1686,7 +1686,7 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B57" t="s">
         <v>14</v>
@@ -1703,7 +1703,7 @@
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B58" t="s">
         <v>14</v>
@@ -1720,7 +1720,7 @@
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B59" t="s">
         <v>14</v>
@@ -1737,7 +1737,7 @@
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B60" t="s">
         <v>14</v>
@@ -1754,7 +1754,7 @@
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B61" t="s">
         <v>14</v>
@@ -1771,7 +1771,7 @@
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B62" t="s">
         <v>6</v>
@@ -1788,7 +1788,7 @@
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B63" t="s">
         <v>14</v>
@@ -1805,7 +1805,7 @@
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B64" t="s">
         <v>14</v>
@@ -1822,7 +1822,7 @@
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B65" t="s">
         <v>6</v>
@@ -1839,7 +1839,7 @@
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B66" t="s">
         <v>6</v>
@@ -1856,7 +1856,7 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B67" t="s">
         <v>14</v>
@@ -1873,7 +1873,7 @@
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B68" t="s">
         <v>14</v>
@@ -1890,7 +1890,7 @@
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B69" t="s">
         <v>14</v>
@@ -1907,7 +1907,7 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B70" t="s">
         <v>14</v>
@@ -1924,7 +1924,7 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B71" t="s">
         <v>14</v>
@@ -1941,7 +1941,7 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B72" t="s">
         <v>14</v>
@@ -1958,7 +1958,7 @@
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B73" t="s">
         <v>14</v>
@@ -1975,7 +1975,7 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B74" t="s">
         <v>14</v>
@@ -1992,7 +1992,7 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B75" t="s">
         <v>14</v>
@@ -2009,7 +2009,7 @@
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B76" t="s">
         <v>14</v>
@@ -2026,7 +2026,7 @@
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B77" t="s">
         <v>14</v>
@@ -2043,7 +2043,7 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B78" t="s">
         <v>14</v>
@@ -2060,7 +2060,7 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B79" t="s">
         <v>14</v>
@@ -2077,7 +2077,7 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B80" t="s">
         <v>14</v>
@@ -2094,7 +2094,7 @@
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B81" t="s">
         <v>14</v>
@@ -2111,7 +2111,7 @@
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B82" t="s">
         <v>14</v>
@@ -2128,7 +2128,7 @@
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B83" t="s">
         <v>14</v>
@@ -2145,7 +2145,7 @@
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B84" t="s">
         <v>14</v>
@@ -2162,7 +2162,7 @@
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B85" t="s">
         <v>14</v>
@@ -2179,7 +2179,7 @@
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B86" t="s">
         <v>14</v>
@@ -2196,7 +2196,7 @@
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B87" t="s">
         <v>14</v>
@@ -2213,7 +2213,7 @@
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B88" t="s">
         <v>14</v>
@@ -2230,7 +2230,7 @@
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B89" t="s">
         <v>14</v>
@@ -2247,7 +2247,7 @@
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B90" t="s">
         <v>14</v>
@@ -2264,7 +2264,7 @@
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B91" t="s">
         <v>14</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B92" t="s">
         <v>14</v>
@@ -2298,7 +2298,7 @@
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B93" t="s">
         <v>14</v>
@@ -2315,7 +2315,7 @@
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B94" t="s">
         <v>14</v>
@@ -2332,7 +2332,7 @@
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B95" t="s">
         <v>14</v>
@@ -2349,7 +2349,7 @@
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B96" t="s">
         <v>14</v>
@@ -2366,7 +2366,7 @@
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B97" t="s">
         <v>14</v>
@@ -2383,7 +2383,7 @@
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B98" t="s">
         <v>14</v>
@@ -2400,7 +2400,7 @@
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B99" t="s">
         <v>14</v>
@@ -2417,7 +2417,7 @@
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B100" t="s">
         <v>14</v>
@@ -2434,7 +2434,7 @@
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B101" t="s">
         <v>14</v>
@@ -2451,7 +2451,7 @@
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B102" t="s">
         <v>14</v>
@@ -2468,7 +2468,7 @@
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B103" t="s">
         <v>14</v>
@@ -2485,7 +2485,7 @@
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B104" t="s">
         <v>14</v>
@@ -2502,7 +2502,7 @@
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B105" t="s">
         <v>14</v>
@@ -2519,7 +2519,7 @@
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B106" t="s">
         <v>14</v>
@@ -2536,7 +2536,7 @@
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B107" t="s">
         <v>14</v>

</xml_diff>